<commit_message>
pull de pc de cg e agora novos proejtos kanban
</commit_message>
<xml_diff>
--- a/batcaverna/planilhas/kanban.xlsx
+++ b/batcaverna/planilhas/kanban.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Projetos" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="190">
   <si>
     <t>Título</t>
   </si>
@@ -118,6 +118,57 @@
     <t>Copa do Mundo 2026</t>
   </si>
   <si>
+    <t>Minicurso Circuitos Eletricos CC</t>
+  </si>
+  <si>
+    <t>Web Developer Javascript (NextJS and NodeJS)</t>
+  </si>
+  <si>
+    <t>Python Developer</t>
+  </si>
+  <si>
+    <t>3 Agentes de AI - Python + N8N</t>
+  </si>
+  <si>
+    <t>AG - UFF - PIBIC</t>
+  </si>
+  <si>
+    <t>Dashboard Website Templates</t>
+  </si>
+  <si>
+    <t>Software Developer - Pyside6 DESKTOP (Estudos)</t>
+  </si>
+  <si>
+    <t>C3PO Gemini</t>
+  </si>
+  <si>
+    <t>CLAUDE CODE</t>
+  </si>
+  <si>
+    <t>Cientista de Dados</t>
+  </si>
+  <si>
+    <t>Meus Projetos Github 2026</t>
+  </si>
+  <si>
+    <t>Pikachu Rest API</t>
+  </si>
+  <si>
+    <t>Quizz App with AI</t>
+  </si>
+  <si>
+    <t>Lista De Tarefas Pendentes</t>
+  </si>
+  <si>
+    <t>Estudos Circuitos CA e Eletromagnetismo (Física 2)</t>
+  </si>
+  <si>
+    <t>Estudos SEP - ONS - AnaRede e Organon</t>
+  </si>
+  <si>
+    <t>Metas e Pautas - Reunião ONS PLC 2026</t>
+  </si>
+  <si>
     <t>in progress</t>
   </si>
   <si>
@@ -145,6 +196,9 @@
     <t>completed</t>
   </si>
   <si>
+    <t>coding</t>
+  </si>
+  <si>
     <t>868d3j5vf</t>
   </si>
   <si>
@@ -226,6 +280,39 @@
     <t>1781658844848</t>
   </si>
   <si>
+    <t>868d3j6h0</t>
+  </si>
+  <si>
+    <t>1764430968647</t>
+  </si>
+  <si>
+    <t>1764440045643</t>
+  </si>
+  <si>
+    <t>1764441187392</t>
+  </si>
+  <si>
+    <t>1765290587715</t>
+  </si>
+  <si>
+    <t>1768308251598</t>
+  </si>
+  <si>
+    <t>1768931860396</t>
+  </si>
+  <si>
+    <t>1770229451483</t>
+  </si>
+  <si>
+    <t>1770652547085</t>
+  </si>
+  <si>
+    <t>1770831420720</t>
+  </si>
+  <si>
+    <t>1770845276516</t>
+  </si>
+  <si>
     <t>uff</t>
   </si>
   <si>
@@ -250,6 +337,12 @@
     <t>spiritual</t>
   </si>
   <si>
+    <t>js</t>
+  </si>
+  <si>
+    <t>web</t>
+  </si>
+  <si>
     <t>09/01/2024</t>
   </si>
   <si>
@@ -307,6 +400,21 @@
     <t>16/06/2026</t>
   </si>
   <si>
+    <t>07/01/2024</t>
+  </si>
+  <si>
+    <t>29/11/2025</t>
+  </si>
+  <si>
+    <t>09/12/2025</t>
+  </si>
+  <si>
+    <t>20/01/2026</t>
+  </si>
+  <si>
+    <t>09/02/2026</t>
+  </si>
+  <si>
     <t>06/07/2026</t>
   </si>
   <si>
@@ -334,6 +442,18 @@
     <t>02/07/2026</t>
   </si>
   <si>
+    <t>24/02/2026</t>
+  </si>
+  <si>
+    <t>27/02/2026</t>
+  </si>
+  <si>
+    <t>26/02/2026</t>
+  </si>
+  <si>
+    <t>17/02/2026</t>
+  </si>
+  <si>
     <t>UFF-Minicurso-Circuitos-Eletricos-CC.md</t>
   </si>
   <si>
@@ -413,6 +533,57 @@
   </si>
   <si>
     <t>Copa-do-Mundo-2026.md</t>
+  </si>
+  <si>
+    <t>Minicurso-Circuitos-Eletricos-CC.md</t>
+  </si>
+  <si>
+    <t>Web-Developer-Javascript-NextJS-and-NodeJS.md</t>
+  </si>
+  <si>
+    <t>Python-Developer.md</t>
+  </si>
+  <si>
+    <t>3-Agentes-de-AI-Python-N8N.md</t>
+  </si>
+  <si>
+    <t>AG-UFF-PIBIC.md</t>
+  </si>
+  <si>
+    <t>Dashboard-Website-Templates.md</t>
+  </si>
+  <si>
+    <t>Software-Developer-Pyside6-DESKTOP-Estudos.md</t>
+  </si>
+  <si>
+    <t>C3PO-Gemini.md</t>
+  </si>
+  <si>
+    <t>CLAUDE-CODE.md</t>
+  </si>
+  <si>
+    <t>Cientista-de-Dados.md</t>
+  </si>
+  <si>
+    <t>Meus-Projetos-Github-2026.md</t>
+  </si>
+  <si>
+    <t>Pikachu-Rest-API.md</t>
+  </si>
+  <si>
+    <t>Quizz-App-with-AI.md</t>
+  </si>
+  <si>
+    <t>Lista-De-Tarefas-Pendentes.md</t>
+  </si>
+  <si>
+    <t>Estudos-Circuitos-CA-e-Eletromagnetismo-Física-2.md</t>
+  </si>
+  <si>
+    <t>Estudos-SEP-ONS-AnaRede-e-Organon.md</t>
+  </si>
+  <si>
+    <t>Metas-e-Pautas-Reunião-ONS-PLC-2026.md</t>
   </si>
 </sst>
 </file>
@@ -770,7 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -801,22 +972,22 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="F2" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G2" t="s">
-        <v>106</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -824,22 +995,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
       <c r="F3" t="s">
-        <v>98</v>
+        <v>134</v>
       </c>
       <c r="G3" t="s">
-        <v>107</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -847,22 +1018,22 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E4" t="s">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="F4" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="G4" t="s">
-        <v>108</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -870,22 +1041,22 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="D5" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E5" t="s">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G5" t="s">
-        <v>109</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -893,22 +1064,22 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="D6" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>113</v>
       </c>
       <c r="F6" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G6" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -916,22 +1087,22 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="D7" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="F7" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
       <c r="G7" t="s">
-        <v>111</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -939,22 +1110,22 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E8" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="F8" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="G8" t="s">
-        <v>112</v>
+        <v>152</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -962,22 +1133,22 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="D9" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="E9" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="F9" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="G9" t="s">
-        <v>113</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -985,22 +1156,22 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="F10" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G10" t="s">
-        <v>114</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1008,22 +1179,22 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="E11" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="F11" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G11" t="s">
-        <v>115</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -1031,22 +1202,22 @@
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="E12" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="F12" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G12" t="s">
-        <v>116</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1054,22 +1225,22 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E13" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="F13" t="s">
-        <v>102</v>
+        <v>138</v>
       </c>
       <c r="G13" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1077,22 +1248,22 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="E14" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="F14" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
       <c r="G14" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1100,22 +1271,22 @@
         <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="D15" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E15" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="F15" t="s">
-        <v>104</v>
+        <v>140</v>
       </c>
       <c r="G15" t="s">
-        <v>119</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1123,22 +1294,22 @@
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="E16" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="F16" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G16" t="s">
-        <v>120</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1146,22 +1317,22 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="C17" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="D17" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E17" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="F17" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
       <c r="G17" t="s">
-        <v>121</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1169,22 +1340,22 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="C18" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="D18" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="E18" t="s">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="F18" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="G18" t="s">
-        <v>122</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1192,22 +1363,22 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="C19" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="E19" t="s">
-        <v>90</v>
+        <v>121</v>
       </c>
       <c r="F19" t="s">
-        <v>105</v>
+        <v>141</v>
       </c>
       <c r="G19" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1215,22 +1386,22 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="D20" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="F20" t="s">
-        <v>105</v>
+        <v>141</v>
       </c>
       <c r="G20" t="s">
-        <v>124</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1238,22 +1409,22 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="D21" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="E21" t="s">
-        <v>91</v>
+        <v>122</v>
       </c>
       <c r="F21" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G21" t="s">
-        <v>125</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1261,22 +1432,22 @@
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E22" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="F22" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G22" t="s">
-        <v>126</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1284,22 +1455,22 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="D23" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E23" t="s">
-        <v>93</v>
+        <v>124</v>
       </c>
       <c r="F23" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
       <c r="G23" t="s">
-        <v>127</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1307,22 +1478,22 @@
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="C24" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="D24" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="E24" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="F24" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
       <c r="G24" t="s">
-        <v>128</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1330,22 +1501,22 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="D25" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E25" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="F25" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="G25" t="s">
-        <v>129</v>
+        <v>169</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1353,22 +1524,22 @@
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="C26" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="D26" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E26" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="F26" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="G26" t="s">
-        <v>130</v>
+        <v>170</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1376,22 +1547,22 @@
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C27" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E27" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="F27" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G27" t="s">
-        <v>131</v>
+        <v>171</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1399,22 +1570,413 @@
         <v>33</v>
       </c>
       <c r="B28" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" t="s">
+        <v>87</v>
+      </c>
+      <c r="D28" t="s">
+        <v>101</v>
+      </c>
+      <c r="E28" t="s">
+        <v>127</v>
+      </c>
+      <c r="F28" t="s">
+        <v>133</v>
+      </c>
+      <c r="G28" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" t="s">
+        <v>99</v>
+      </c>
+      <c r="E29" t="s">
+        <v>109</v>
+      </c>
+      <c r="F29" t="s">
+        <v>142</v>
+      </c>
+      <c r="G29" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" t="s">
+        <v>107</v>
+      </c>
+      <c r="E30" t="s">
+        <v>128</v>
+      </c>
+      <c r="F30" t="s">
+        <v>142</v>
+      </c>
+      <c r="G30" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" t="s">
+        <v>63</v>
+      </c>
+      <c r="D31" t="s">
+        <v>101</v>
+      </c>
+      <c r="E31" t="s">
+        <v>111</v>
+      </c>
+      <c r="F31" t="s">
+        <v>135</v>
+      </c>
+      <c r="G31" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" t="s">
+        <v>100</v>
+      </c>
+      <c r="E32" t="s">
+        <v>129</v>
+      </c>
+      <c r="F32" t="s">
+        <v>142</v>
+      </c>
+      <c r="G32" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" t="s">
         <v>38</v>
       </c>
-      <c r="C28" t="s">
-        <v>69</v>
-      </c>
-      <c r="D28" t="s">
-        <v>72</v>
-      </c>
-      <c r="E28" t="s">
+      <c r="B33" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" t="s">
+        <v>90</v>
+      </c>
+      <c r="D33" t="s">
+        <v>99</v>
+      </c>
+      <c r="E33" t="s">
+        <v>129</v>
+      </c>
+      <c r="F33" t="s">
+        <v>143</v>
+      </c>
+      <c r="G33" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D34" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" t="s">
+        <v>129</v>
+      </c>
+      <c r="F34" t="s">
+        <v>142</v>
+      </c>
+      <c r="G34" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" t="s">
+        <v>51</v>
+      </c>
+      <c r="C35" t="s">
+        <v>92</v>
+      </c>
+      <c r="D35" t="s">
+        <v>100</v>
+      </c>
+      <c r="E35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F35" t="s">
+        <v>142</v>
+      </c>
+      <c r="G35" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36" t="s">
+        <v>58</v>
+      </c>
+      <c r="C36" t="s">
+        <v>93</v>
+      </c>
+      <c r="D36" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" t="s">
+        <v>114</v>
+      </c>
+      <c r="F36" t="s">
+        <v>132</v>
+      </c>
+      <c r="G36" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" t="s">
+        <v>68</v>
+      </c>
+      <c r="D37" t="s">
+        <v>105</v>
+      </c>
+      <c r="E37" t="s">
+        <v>114</v>
+      </c>
+      <c r="F37" t="s">
+        <v>142</v>
+      </c>
+      <c r="G37" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C38" t="s">
+        <v>70</v>
+      </c>
+      <c r="D38" t="s">
+        <v>105</v>
+      </c>
+      <c r="E38" t="s">
+        <v>115</v>
+      </c>
+      <c r="F38" t="s">
+        <v>143</v>
+      </c>
+      <c r="G38" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39" t="s">
+        <v>60</v>
+      </c>
+      <c r="C39" t="s">
+        <v>94</v>
+      </c>
+      <c r="D39" t="s">
+        <v>100</v>
+      </c>
+      <c r="E39" t="s">
+        <v>131</v>
+      </c>
+      <c r="F39" t="s">
+        <v>117</v>
+      </c>
+      <c r="G39" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" t="s">
+        <v>45</v>
+      </c>
+      <c r="B40" t="s">
+        <v>59</v>
+      </c>
+      <c r="C40" t="s">
+        <v>95</v>
+      </c>
+      <c r="D40" t="s">
+        <v>100</v>
+      </c>
+      <c r="E40" t="s">
+        <v>116</v>
+      </c>
+      <c r="F40" t="s">
+        <v>117</v>
+      </c>
+      <c r="G40" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" t="s">
+        <v>59</v>
+      </c>
+      <c r="C41" t="s">
+        <v>71</v>
+      </c>
+      <c r="D41" t="s">
+        <v>102</v>
+      </c>
+      <c r="E41" t="s">
+        <v>116</v>
+      </c>
+      <c r="F41" t="s">
+        <v>116</v>
+      </c>
+      <c r="G41" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" t="s">
         <v>96</v>
       </c>
-      <c r="F28" t="s">
+      <c r="D42" t="s">
+        <v>102</v>
+      </c>
+      <c r="E42" t="s">
+        <v>132</v>
+      </c>
+      <c r="F42" t="s">
+        <v>143</v>
+      </c>
+      <c r="G42" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43" t="s">
+        <v>57</v>
+      </c>
+      <c r="C43" t="s">
+        <v>73</v>
+      </c>
+      <c r="D43" t="s">
+        <v>101</v>
+      </c>
+      <c r="E43" t="s">
+        <v>117</v>
+      </c>
+      <c r="F43" t="s">
+        <v>142</v>
+      </c>
+      <c r="G43" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" t="s">
+        <v>49</v>
+      </c>
+      <c r="B44" t="s">
+        <v>58</v>
+      </c>
+      <c r="C44" t="s">
         <v>97</v>
       </c>
-      <c r="G28" t="s">
-        <v>132</v>
+      <c r="D44" t="s">
+        <v>101</v>
+      </c>
+      <c r="E44" t="s">
+        <v>117</v>
+      </c>
+      <c r="F44" t="s">
+        <v>144</v>
+      </c>
+      <c r="G44" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" t="s">
+        <v>50</v>
+      </c>
+      <c r="B45" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" t="s">
+        <v>98</v>
+      </c>
+      <c r="D45" t="s">
+        <v>101</v>
+      </c>
+      <c r="E45" t="s">
+        <v>117</v>
+      </c>
+      <c r="F45" t="s">
+        <v>145</v>
+      </c>
+      <c r="G45" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>